<commit_message>
Sozialversicherungsakten: Tabellenlayout und Downloads verfeinern (v445.16.2) (#460)
</commit_message>
<xml_diff>
--- a/testakten/sozialversicherung-programmierer-leipzig/27_Rechnungsabgleich_2025.xlsx
+++ b/testakten/sozialversicherung-programmierer-leipzig/27_Rechnungsabgleich_2025.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nordlicht 2025" sheetId="1" r:id="Rbb482b6e4fa94222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linde und Gesamt" sheetId="2" r:id="R4b2b4c26ce164673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nordlicht 2025" sheetId="1" r:id="R3e92909994f24c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linde und Gesamt" sheetId="2" r:id="R91283b14246a47ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,8 +14,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="#,##0.00 &quot;€&quot;;[Red](#,##0.00) &quot;€&quot;;&quot;–&quot;"/>
+    <x:numFmt numFmtId="201" formatCode="0&quot;  &quot;"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0.00 &quot;€  &quot;;[Red](#,##0.00) &quot;€  &quot;;&quot;–  &quot;"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -79,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -90,14 +92,68 @@
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -349,384 +405,384 @@
       <x:c r="H3" s="1"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="7" t="str">
-        <x:v>Leistungsmonat</x:v>
-      </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Monat</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
         <x:v>Stunden</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="str">
+      <x:c r="C4" s="10" t="str">
         <x:v>Satz netto</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="str">
+      <x:c r="D4" s="10" t="str">
         <x:v>Nettohonorar</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="str">
+      <x:c r="E4" s="10" t="str">
         <x:v>USt 19 %</x:v>
       </x:c>
-      <x:c r="F4" s="7" t="str">
+      <x:c r="F4" s="10" t="str">
         <x:v>Bruttobetrag</x:v>
       </x:c>
-      <x:c r="G4" s="7" t="str">
+      <x:c r="G4" s="10" t="str">
         <x:v>Zahlungseingang</x:v>
       </x:c>
-      <x:c r="H4" s="7" t="str">
+      <x:c r="H4" s="8" t="str">
         <x:v>Bemerkung</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="1" t="str">
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="9" t="str">
         <x:v>2025-01</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="n">
+      <x:c r="B5" s="23" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="n">
+      <x:c r="C5" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D5" s="10" t="n">
+      <x:c r="D5" s="26" t="n">
         <x:f>B5*C5</x:f>
         <x:v>13440</x:v>
       </x:c>
-      <x:c r="E5" s="10" t="n">
+      <x:c r="E5" s="26" t="n">
         <x:f>ROUND(D5*19%,2)</x:f>
         <x:v>2553.6</x:v>
       </x:c>
-      <x:c r="F5" s="10" t="n">
+      <x:c r="F5" s="26" t="n">
         <x:f>D5+E5</x:f>
         <x:v>15993.6</x:v>
       </x:c>
-      <x:c r="G5" s="1" t="str">
+      <x:c r="G5" s="28" t="str">
         <x:v>2025-02-26</x:v>
       </x:c>
-      <x:c r="H5" s="14" t="str"/>
-    </x:row>
-    <x:row r="6" ht="34" customHeight="1">
-      <x:c r="A6" s="1" t="str">
+      <x:c r="H5" s="17" t="str"/>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="9" t="str">
         <x:v>2025-02</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="n">
+      <x:c r="B6" s="23" t="n">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="C6" s="13" t="n">
+      <x:c r="C6" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D6" s="10" t="n">
+      <x:c r="D6" s="26" t="n">
         <x:f>B6*C6</x:f>
         <x:v>14280</x:v>
       </x:c>
-      <x:c r="E6" s="10" t="n">
+      <x:c r="E6" s="26" t="n">
         <x:f>ROUND(D6*19%,2)</x:f>
         <x:v>2713.2</x:v>
       </x:c>
-      <x:c r="F6" s="10" t="n">
+      <x:c r="F6" s="26" t="n">
         <x:f>D6+E6</x:f>
         <x:v>16993.2</x:v>
       </x:c>
-      <x:c r="G6" s="1" t="str">
+      <x:c r="G6" s="28" t="str">
         <x:v>2025-03-26</x:v>
       </x:c>
-      <x:c r="H6" s="14" t="str"/>
-    </x:row>
-    <x:row r="7" ht="34" customHeight="1">
-      <x:c r="A7" s="1" t="str">
+      <x:c r="H6" s="17" t="str"/>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="9" t="str">
         <x:v>2025-03</x:v>
       </x:c>
-      <x:c r="B7" s="12" t="n">
+      <x:c r="B7" s="23" t="n">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="C7" s="13" t="n">
+      <x:c r="C7" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D7" s="10" t="n">
+      <x:c r="D7" s="26" t="n">
         <x:f>B7*C7</x:f>
         <x:v>15120</x:v>
       </x:c>
-      <x:c r="E7" s="10" t="n">
+      <x:c r="E7" s="26" t="n">
         <x:f>ROUND(D7*19%,2)</x:f>
         <x:v>2872.8</x:v>
       </x:c>
-      <x:c r="F7" s="10" t="n">
+      <x:c r="F7" s="26" t="n">
         <x:f>D7+E7</x:f>
         <x:v>17992.8</x:v>
       </x:c>
-      <x:c r="G7" s="1" t="str">
+      <x:c r="G7" s="28" t="str">
         <x:v>2025-04-25</x:v>
       </x:c>
-      <x:c r="H7" s="14" t="str"/>
-    </x:row>
-    <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="1" t="str">
+      <x:c r="H7" s="17" t="str"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="9" t="str">
         <x:v>2025-04</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="n">
+      <x:c r="B8" s="23" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="C8" s="13" t="n">
+      <x:c r="C8" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D8" s="10" t="n">
+      <x:c r="D8" s="26" t="n">
         <x:f>B8*C8</x:f>
         <x:v>12600</x:v>
       </x:c>
-      <x:c r="E8" s="10" t="n">
+      <x:c r="E8" s="26" t="n">
         <x:f>ROUND(D8*19%,2)</x:f>
         <x:v>2394</x:v>
       </x:c>
-      <x:c r="F8" s="10" t="n">
+      <x:c r="F8" s="26" t="n">
         <x:f>D8+E8</x:f>
         <x:v>14994</x:v>
       </x:c>
-      <x:c r="G8" s="1" t="str">
+      <x:c r="G8" s="28" t="str">
         <x:v>2025-05-26</x:v>
       </x:c>
-      <x:c r="H8" s="14" t="str">
+      <x:c r="H8" s="17" t="str">
         <x:v>3 Stunden nach Rücksprache abgezogen</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="1" t="str">
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="9" t="str">
         <x:v>2025-05</x:v>
       </x:c>
-      <x:c r="B9" s="12" t="n">
+      <x:c r="B9" s="23" t="n">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="C9" s="13" t="n">
+      <x:c r="C9" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D9" s="10" t="n">
+      <x:c r="D9" s="26" t="n">
         <x:f>B9*C9</x:f>
         <x:v>14280</x:v>
       </x:c>
-      <x:c r="E9" s="10" t="n">
+      <x:c r="E9" s="26" t="n">
         <x:f>ROUND(D9*19%,2)</x:f>
         <x:v>2713.2</x:v>
       </x:c>
-      <x:c r="F9" s="10" t="n">
+      <x:c r="F9" s="26" t="n">
         <x:f>D9+E9</x:f>
         <x:v>16993.2</x:v>
       </x:c>
-      <x:c r="G9" s="1" t="str">
+      <x:c r="G9" s="28" t="str">
         <x:v>2025-06-26</x:v>
       </x:c>
-      <x:c r="H9" s="14" t="str"/>
-    </x:row>
-    <x:row r="10" ht="34" customHeight="1">
-      <x:c r="A10" s="1" t="str">
+      <x:c r="H9" s="17" t="str"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="9" t="str">
         <x:v>2025-06</x:v>
       </x:c>
-      <x:c r="B10" s="12" t="n">
+      <x:c r="B10" s="23" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="C10" s="13" t="n">
+      <x:c r="C10" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D10" s="10" t="n">
+      <x:c r="D10" s="26" t="n">
         <x:f>B10*C10</x:f>
         <x:v>13440</x:v>
       </x:c>
-      <x:c r="E10" s="10" t="n">
+      <x:c r="E10" s="26" t="n">
         <x:f>ROUND(D10*19%,2)</x:f>
         <x:v>2553.6</x:v>
       </x:c>
-      <x:c r="F10" s="10" t="n">
+      <x:c r="F10" s="26" t="n">
         <x:f>D10+E10</x:f>
         <x:v>15993.6</x:v>
       </x:c>
-      <x:c r="G10" s="1" t="str">
+      <x:c r="G10" s="28" t="str">
         <x:v>2025-07-25</x:v>
       </x:c>
-      <x:c r="H10" s="14" t="str"/>
-    </x:row>
-    <x:row r="11" ht="34" customHeight="1">
-      <x:c r="A11" s="1" t="str">
+      <x:c r="H10" s="17" t="str"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="9" t="str">
         <x:v>2025-07</x:v>
       </x:c>
-      <x:c r="B11" s="12" t="n">
+      <x:c r="B11" s="23" t="n">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="C11" s="13" t="n">
+      <x:c r="C11" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D11" s="10" t="n">
+      <x:c r="D11" s="26" t="n">
         <x:f>B11*C11</x:f>
         <x:v>10080</x:v>
       </x:c>
-      <x:c r="E11" s="10" t="n">
+      <x:c r="E11" s="26" t="n">
         <x:f>ROUND(D11*19%,2)</x:f>
         <x:v>1915.2</x:v>
       </x:c>
-      <x:c r="F11" s="10" t="n">
+      <x:c r="F11" s="26" t="n">
         <x:f>D11+E11</x:f>
         <x:v>11995.2</x:v>
       </x:c>
-      <x:c r="G11" s="1" t="str">
+      <x:c r="G11" s="28" t="str">
         <x:v>2025-08-26</x:v>
       </x:c>
-      <x:c r="H11" s="14" t="str">
+      <x:c r="H11" s="17" t="str">
         <x:v>Zwei Wochen ohne Leistungsstunden</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="1" t="str">
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="9" t="str">
         <x:v>2025-08</x:v>
       </x:c>
-      <x:c r="B12" s="12" t="n">
+      <x:c r="B12" s="23" t="n">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="C12" s="13" t="n">
+      <x:c r="C12" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D12" s="10" t="n">
+      <x:c r="D12" s="26" t="n">
         <x:f>B12*C12</x:f>
         <x:v>11760</x:v>
       </x:c>
-      <x:c r="E12" s="10" t="n">
+      <x:c r="E12" s="26" t="n">
         <x:f>ROUND(D12*19%,2)</x:f>
         <x:v>2234.4</x:v>
       </x:c>
-      <x:c r="F12" s="10" t="n">
+      <x:c r="F12" s="26" t="n">
         <x:f>D12+E12</x:f>
         <x:v>13994.4</x:v>
       </x:c>
-      <x:c r="G12" s="1" t="str">
+      <x:c r="G12" s="28" t="str">
         <x:v>2025-09-26</x:v>
       </x:c>
-      <x:c r="H12" s="14" t="str"/>
-    </x:row>
-    <x:row r="13" ht="34" customHeight="1">
-      <x:c r="A13" s="1" t="str">
+      <x:c r="H12" s="17" t="str"/>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="9" t="str">
         <x:v>2025-09</x:v>
       </x:c>
-      <x:c r="B13" s="12" t="n">
+      <x:c r="B13" s="23" t="n">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="C13" s="13" t="n">
+      <x:c r="C13" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D13" s="10" t="n">
+      <x:c r="D13" s="26" t="n">
         <x:f>B13*C13</x:f>
         <x:v>15120</x:v>
       </x:c>
-      <x:c r="E13" s="10" t="n">
+      <x:c r="E13" s="26" t="n">
         <x:f>ROUND(D13*19%,2)</x:f>
         <x:v>2872.8</x:v>
       </x:c>
-      <x:c r="F13" s="10" t="n">
+      <x:c r="F13" s="26" t="n">
         <x:f>D13+E13</x:f>
         <x:v>17992.8</x:v>
       </x:c>
-      <x:c r="G13" s="1" t="str">
+      <x:c r="G13" s="28" t="str">
         <x:v>2025-10-27</x:v>
       </x:c>
-      <x:c r="H13" s="14" t="str"/>
-    </x:row>
-    <x:row r="14" ht="34" customHeight="1">
-      <x:c r="A14" s="1" t="str">
+      <x:c r="H13" s="17" t="str"/>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="9" t="str">
         <x:v>2025-10</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="n">
+      <x:c r="B14" s="23" t="n">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="C14" s="13" t="n">
+      <x:c r="C14" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D14" s="10" t="n">
+      <x:c r="D14" s="26" t="n">
         <x:f>B14*C14</x:f>
         <x:v>15960</x:v>
       </x:c>
-      <x:c r="E14" s="10" t="n">
+      <x:c r="E14" s="26" t="n">
         <x:f>ROUND(D14*19%,2)</x:f>
         <x:v>3032.4</x:v>
       </x:c>
-      <x:c r="F14" s="10" t="n">
+      <x:c r="F14" s="26" t="n">
         <x:f>D14+E14</x:f>
         <x:v>18992.4</x:v>
       </x:c>
-      <x:c r="G14" s="1" t="str">
+      <x:c r="G14" s="28" t="str">
         <x:v>2025-11-26</x:v>
       </x:c>
-      <x:c r="H14" s="14" t="str"/>
-    </x:row>
-    <x:row r="15" ht="34" customHeight="1">
-      <x:c r="A15" s="1" t="str">
+      <x:c r="H14" s="17" t="str"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="9" t="str">
         <x:v>2025-11</x:v>
       </x:c>
-      <x:c r="B15" s="12" t="n">
+      <x:c r="B15" s="23" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="C15" s="13" t="n">
+      <x:c r="C15" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D15" s="10" t="n">
+      <x:c r="D15" s="26" t="n">
         <x:f>B15*C15</x:f>
         <x:v>13440</x:v>
       </x:c>
-      <x:c r="E15" s="10" t="n">
+      <x:c r="E15" s="26" t="n">
         <x:f>ROUND(D15*19%,2)</x:f>
         <x:v>2553.6</x:v>
       </x:c>
-      <x:c r="F15" s="10" t="n">
+      <x:c r="F15" s="26" t="n">
         <x:f>D15+E15</x:f>
         <x:v>15993.6</x:v>
       </x:c>
-      <x:c r="G15" s="1" t="str">
+      <x:c r="G15" s="28" t="str">
         <x:v>2025-12-23</x:v>
       </x:c>
-      <x:c r="H15" s="14" t="str"/>
-    </x:row>
-    <x:row r="16" ht="34" customHeight="1">
-      <x:c r="A16" s="1" t="str">
+      <x:c r="H15" s="17" t="str"/>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="9" t="str">
         <x:v>2025-12</x:v>
       </x:c>
-      <x:c r="B16" s="12" t="n">
+      <x:c r="B16" s="23" t="n">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="C16" s="13" t="n">
+      <x:c r="C16" s="25" t="n">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="D16" s="10" t="n">
+      <x:c r="D16" s="26" t="n">
         <x:f>B16*C16</x:f>
         <x:v>9240</x:v>
       </x:c>
-      <x:c r="E16" s="10" t="n">
+      <x:c r="E16" s="26" t="n">
         <x:f>ROUND(D16*19%,2)</x:f>
         <x:v>1755.6</x:v>
       </x:c>
-      <x:c r="F16" s="10" t="n">
+      <x:c r="F16" s="26" t="n">
         <x:f>D16+E16</x:f>
         <x:v>10995.6</x:v>
       </x:c>
-      <x:c r="G16" s="1" t="str">
+      <x:c r="G16" s="28" t="str">
         <x:v>2026-01-26</x:v>
       </x:c>
-      <x:c r="H16" s="14" t="str">
+      <x:c r="H16" s="17" t="str">
         <x:v>Zahlung erst im Folgejahr</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="28" customHeight="1">
-      <x:c r="A17" s="9" t="str">
+      <x:c r="A17" s="12" t="str">
         <x:v>Summe</x:v>
       </x:c>
-      <x:c r="B17" s="9" t="n">
+      <x:c r="B17" s="24" t="n">
         <x:f>SUM(B5:B16)</x:f>
         <x:v>1512</x:v>
       </x:c>
-      <x:c r="C17" s="11"/>
-      <x:c r="D17" s="11" t="n">
+      <x:c r="C17" s="27"/>
+      <x:c r="D17" s="27" t="n">
         <x:f>SUM(D5:D16)</x:f>
         <x:v>158760</x:v>
       </x:c>
-      <x:c r="E17" s="11" t="n">
+      <x:c r="E17" s="27" t="n">
         <x:f>SUM(E5:E16)</x:f>
         <x:v>30164.399999999998</x:v>
       </x:c>
-      <x:c r="F17" s="11" t="n">
+      <x:c r="F17" s="27" t="n">
         <x:f>SUM(F5:F16)</x:f>
         <x:v>188924.4</x:v>
       </x:c>
-      <x:c r="G17" s="9"/>
-      <x:c r="H17" s="9"/>
+      <x:c r="G17" s="12"/>
+      <x:c r="H17" s="12"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="1"/>
@@ -738,41 +794,41 @@
       <x:c r="G18" s="1"/>
       <x:c r="H18" s="1"/>
     </x:row>
-    <x:row r="19" ht="34" customHeight="1">
-      <x:c r="A19" s="15" t="str">
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="29" t="str">
         <x:v>Nur Nordlicht-Rechnungen für Leistungen 2025. Die ursprüngliche Migration wurde 2024 mit 95 € pro Stunde abgerechnet.</x:v>
       </x:c>
-      <x:c r="B19" s="15"/>
-      <x:c r="C19" s="15"/>
-      <x:c r="D19" s="15"/>
-      <x:c r="E19" s="15"/>
-      <x:c r="F19" s="15"/>
-      <x:c r="G19" s="15"/>
-      <x:c r="H19" s="15"/>
-    </x:row>
-    <x:row r="20" ht="34" customHeight="1">
-      <x:c r="A20" s="15" t="str">
+      <x:c r="B19" s="29"/>
+      <x:c r="C19" s="29"/>
+      <x:c r="D19" s="29"/>
+      <x:c r="E19" s="29"/>
+      <x:c r="F19" s="29"/>
+      <x:c r="G19" s="29"/>
+      <x:c r="H19" s="29"/>
+    </x:row>
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="29" t="str">
         <x:v>Zahlungsdaten stammen aus den Kontozuordnungen. Die Dezemberleistung wurde erst am 26.01.2026 bezahlt.</x:v>
       </x:c>
-      <x:c r="B20" s="15"/>
-      <x:c r="C20" s="15"/>
-      <x:c r="D20" s="15"/>
-      <x:c r="E20" s="15"/>
-      <x:c r="F20" s="15"/>
-      <x:c r="G20" s="15"/>
-      <x:c r="H20" s="15"/>
-    </x:row>
-    <x:row r="21" ht="34" customHeight="1">
-      <x:c r="A21" s="15" t="str">
+      <x:c r="B20" s="29"/>
+      <x:c r="C20" s="29"/>
+      <x:c r="D20" s="29"/>
+      <x:c r="E20" s="29"/>
+      <x:c r="F20" s="29"/>
+      <x:c r="G20" s="29"/>
+      <x:c r="H20" s="29"/>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="29" t="str">
         <x:v>Rechnung KS-2025-002: Januar 128 Stunden × 105 € = 13.440 € netto; 15.993,60 € brutto.</x:v>
       </x:c>
-      <x:c r="B21" s="15"/>
-      <x:c r="C21" s="15"/>
-      <x:c r="D21" s="15"/>
-      <x:c r="E21" s="15"/>
-      <x:c r="F21" s="15"/>
-      <x:c r="G21" s="15"/>
-      <x:c r="H21" s="15"/>
+      <x:c r="B21" s="29"/>
+      <x:c r="C21" s="29"/>
+      <x:c r="D21" s="29"/>
+      <x:c r="E21" s="29"/>
+      <x:c r="F21" s="29"/>
+      <x:c r="G21" s="29"/>
+      <x:c r="H21" s="29"/>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="1"/>
@@ -847,185 +903,185 @@
       <x:c r="F3" s="1"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="7" t="str">
+      <x:c r="A4" s="8" t="str">
         <x:v>Rechnung / Monat</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="B4" s="10" t="str">
         <x:v>Netto</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="str">
+      <x:c r="C4" s="10" t="str">
         <x:v>USt 19 %</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="str">
+      <x:c r="D4" s="10" t="str">
         <x:v>Brutto</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="str">
+      <x:c r="E4" s="10" t="str">
         <x:v>Zahlung</x:v>
       </x:c>
-      <x:c r="F4" s="7" t="str">
+      <x:c r="F4" s="8" t="str">
         <x:v>Leistung</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
-      <x:c r="A5" s="1" t="str">
+      <x:c r="A5" s="9" t="str">
         <x:v>März 2025</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="n">
+      <x:c r="B5" s="25" t="n">
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="C5" s="10" t="n">
+      <x:c r="C5" s="26" t="n">
         <x:f>ROUND(B5*19%,2)</x:f>
         <x:v>760</x:v>
       </x:c>
-      <x:c r="D5" s="10" t="n">
+      <x:c r="D5" s="26" t="n">
         <x:f>B5+C5</x:f>
         <x:v>4760</x:v>
       </x:c>
-      <x:c r="E5" s="1" t="str">
+      <x:c r="E5" s="28" t="str">
         <x:v>2025-04-09</x:v>
       </x:c>
-      <x:c r="F5" s="14" t="str">
+      <x:c r="F5" s="17" t="str">
         <x:v>Messdatenformat A</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
-      <x:c r="A6" s="1" t="str">
+      <x:c r="A6" s="9" t="str">
         <x:v>Juni 2025</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="n">
+      <x:c r="B6" s="25" t="n">
         <x:v>4800</x:v>
       </x:c>
-      <x:c r="C6" s="10" t="n">
+      <x:c r="C6" s="26" t="n">
         <x:f>ROUND(B6*19%,2)</x:f>
         <x:v>912</x:v>
       </x:c>
-      <x:c r="D6" s="10" t="n">
+      <x:c r="D6" s="26" t="n">
         <x:f>B6+C6</x:f>
         <x:v>5712</x:v>
       </x:c>
-      <x:c r="E6" s="1" t="str">
+      <x:c r="E6" s="28" t="str">
         <x:v>2025-07-08</x:v>
       </x:c>
-      <x:c r="F6" s="14" t="str">
+      <x:c r="F6" s="17" t="str">
         <x:v>Bericht und Prüflauf</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
-      <x:c r="A7" s="1" t="str">
+      <x:c r="A7" s="9" t="str">
         <x:v>September 2025</x:v>
       </x:c>
-      <x:c r="B7" s="13" t="n">
+      <x:c r="B7" s="25" t="n">
         <x:v>5200</x:v>
       </x:c>
-      <x:c r="C7" s="10" t="n">
+      <x:c r="C7" s="26" t="n">
         <x:f>ROUND(B7*19%,2)</x:f>
         <x:v>988</x:v>
       </x:c>
-      <x:c r="D7" s="10" t="n">
+      <x:c r="D7" s="26" t="n">
         <x:f>B7+C7</x:f>
         <x:v>6188</x:v>
       </x:c>
-      <x:c r="E7" s="1" t="str">
+      <x:c r="E7" s="28" t="str">
         <x:v>2025-10-10</x:v>
       </x:c>
-      <x:c r="F7" s="14" t="str">
+      <x:c r="F7" s="17" t="str">
         <x:v>Erweiterung Serienimport</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
-      <x:c r="A8" s="1" t="str">
+      <x:c r="A8" s="9" t="str">
         <x:v>November 2025</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="n">
+      <x:c r="B8" s="25" t="n">
         <x:v>4400</x:v>
       </x:c>
-      <x:c r="C8" s="10" t="n">
+      <x:c r="C8" s="26" t="n">
         <x:f>ROUND(B8*19%,2)</x:f>
         <x:v>836</x:v>
       </x:c>
-      <x:c r="D8" s="10" t="n">
+      <x:c r="D8" s="26" t="n">
         <x:f>B8+C8</x:f>
         <x:v>5236</x:v>
       </x:c>
-      <x:c r="E8" s="1" t="str">
+      <x:c r="E8" s="28" t="str">
         <x:v>2025-12-09</x:v>
       </x:c>
-      <x:c r="F8" s="14" t="str">
+      <x:c r="F8" s="17" t="str">
         <x:v>Zusätzliche Spalten / KS-2025-024</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="1"/>
-      <x:c r="B9" s="10"/>
-      <x:c r="C9" s="10"/>
-      <x:c r="D9" s="10"/>
-      <x:c r="E9" s="1"/>
-      <x:c r="F9" s="1"/>
+      <x:c r="A9" s="9"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
+      <x:c r="E9" s="9"/>
+      <x:c r="F9" s="9"/>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="9" t="str">
+      <x:c r="A10" s="12" t="str">
         <x:v>Linde 2025</x:v>
       </x:c>
-      <x:c r="B10" s="11" t="n">
+      <x:c r="B10" s="27" t="n">
         <x:f>SUM(B5:B8)</x:f>
         <x:v>18400</x:v>
       </x:c>
-      <x:c r="C10" s="11" t="n">
+      <x:c r="C10" s="27" t="n">
         <x:f>SUM(C5:C8)</x:f>
         <x:v>3496</x:v>
       </x:c>
-      <x:c r="D10" s="11" t="n">
+      <x:c r="D10" s="27" t="n">
         <x:f>SUM(D5:D8)</x:f>
         <x:v>21896</x:v>
       </x:c>
-      <x:c r="E10" s="9"/>
-      <x:c r="F10" s="9"/>
+      <x:c r="E10" s="12"/>
+      <x:c r="F10" s="12"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="1"/>
-      <x:c r="B11" s="10"/>
-      <x:c r="C11" s="10"/>
-      <x:c r="D11" s="10"/>
-      <x:c r="E11" s="1"/>
-      <x:c r="F11" s="1"/>
+      <x:c r="A11" s="9"/>
+      <x:c r="B11" s="26"/>
+      <x:c r="C11" s="26"/>
+      <x:c r="D11" s="26"/>
+      <x:c r="E11" s="9"/>
+      <x:c r="F11" s="9"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="1" t="str">
+      <x:c r="A12" s="9" t="str">
         <x:v>Nordlicht 2025</x:v>
       </x:c>
-      <x:c r="B12" s="10" t="n">
+      <x:c r="B12" s="26" t="n">
         <x:f>'Nordlicht 2025'!D17</x:f>
         <x:v>158760</x:v>
       </x:c>
-      <x:c r="C12" s="10" t="n">
+      <x:c r="C12" s="26" t="n">
         <x:f>'Nordlicht 2025'!E17</x:f>
         <x:v>30164.399999999998</x:v>
       </x:c>
-      <x:c r="D12" s="10" t="n">
+      <x:c r="D12" s="26" t="n">
         <x:f>'Nordlicht 2025'!F17</x:f>
         <x:v>188924.4</x:v>
       </x:c>
-      <x:c r="E12" s="1"/>
-      <x:c r="F12" s="1"/>
+      <x:c r="E12" s="9"/>
+      <x:c r="F12" s="9"/>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="9" t="str">
+      <x:c r="A13" s="12" t="str">
         <x:v>Zusammen</x:v>
       </x:c>
-      <x:c r="B13" s="11" t="n">
+      <x:c r="B13" s="27" t="n">
         <x:f>B10+B12</x:f>
         <x:v>177160</x:v>
       </x:c>
-      <x:c r="C13" s="11" t="n">
+      <x:c r="C13" s="27" t="n">
         <x:f>C10+C12</x:f>
         <x:v>33660.399999999994</x:v>
       </x:c>
-      <x:c r="D13" s="11" t="n">
+      <x:c r="D13" s="27" t="n">
         <x:f>D10+D12</x:f>
         <x:v>210820.4</x:v>
       </x:c>
-      <x:c r="E13" s="9"/>
-      <x:c r="F13" s="9"/>
+      <x:c r="E13" s="12"/>
+      <x:c r="F13" s="12"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="1"/>
@@ -1044,24 +1100,24 @@
       <x:c r="F15" s="1"/>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
-      <x:c r="A16" s="15" t="str">
+      <x:c r="A16" s="29" t="str">
         <x:v>Die Aufstellung enthält Umsätze vor Ausgaben. Software, Haftpflicht, Reisen und eigene Vorsorge sind nicht abgezogen.</x:v>
       </x:c>
-      <x:c r="B16" s="15"/>
-      <x:c r="C16" s="15"/>
-      <x:c r="D16" s="15"/>
-      <x:c r="E16" s="15"/>
-      <x:c r="F16" s="15"/>
+      <x:c r="B16" s="29"/>
+      <x:c r="C16" s="29"/>
+      <x:c r="D16" s="29"/>
+      <x:c r="E16" s="29"/>
+      <x:c r="F16" s="29"/>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
-      <x:c r="A17" s="15" t="str">
+      <x:c r="A17" s="29" t="str">
         <x:v>Die Linde-Pakete wurden zum Festpreis angeboten. Stunden für diese Arbeiten werden in der Nordlicht-Liste nicht erfasst.</x:v>
       </x:c>
-      <x:c r="B17" s="15"/>
-      <x:c r="C17" s="15"/>
-      <x:c r="D17" s="15"/>
-      <x:c r="E17" s="15"/>
-      <x:c r="F17" s="15"/>
+      <x:c r="B17" s="29"/>
+      <x:c r="C17" s="29"/>
+      <x:c r="D17" s="29"/>
+      <x:c r="E17" s="29"/>
+      <x:c r="F17" s="29"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="1"/>

</xml_diff>